<commit_message>
all steps in Stock_trading_processes.docx described  yet is covered in this system.
</commit_message>
<xml_diff>
--- a/ORDER_MGMT/regular_order_mgmt/PENDING_ORDERS_REPOSITORY_FILES/Result_Executed_OrderBook_14to24july2026.xlsx
+++ b/ORDER_MGMT/regular_order_mgmt/PENDING_ORDERS_REPOSITORY_FILES/Result_Executed_OrderBook_14to24july2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\python\stocks\ORDER_MGMT\regular_order_mgmt\PENDING_ORDERS_REPOSITORY_FILES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C5F531BA-7FA7-4907-9490-8BAC7743FEF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6E68CC-7D67-4239-A6E4-FD108EF93969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All_Backups" sheetId="2" r:id="rId1"/>
@@ -6049,6 +6049,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BDEAB589-59D4-402D-A28C-AA7262E65C2C}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:G245"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -6080,7 +6081,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>1</v>
       </c>
@@ -6100,7 +6101,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A3" s="4" t="s">
         <v>123</v>
       </c>
@@ -6123,7 +6124,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4" t="s">
         <v>147</v>
       </c>
@@ -6146,7 +6147,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A5" s="4" t="s">
         <v>147</v>
       </c>
@@ -6169,7 +6170,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A6" s="4" t="s">
         <v>168</v>
       </c>
@@ -6192,7 +6193,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A7" s="4"/>
       <c r="B7" s="6"/>
       <c r="C7" s="6"/>
@@ -6201,7 +6202,7 @@
       <c r="F7" s="4"/>
       <c r="G7" s="6"/>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A8" s="4" t="s">
         <v>1</v>
       </c>
@@ -6221,7 +6222,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A9" s="4" t="s">
         <v>123</v>
       </c>
@@ -6244,7 +6245,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A10" s="4" t="s">
         <v>157</v>
       </c>
@@ -6267,7 +6268,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A11" s="4"/>
       <c r="B11" s="5"/>
       <c r="C11" s="5"/>
@@ -6276,7 +6277,7 @@
       <c r="F11" s="4"/>
       <c r="G11" s="5"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A12" s="4" t="s">
         <v>112</v>
       </c>
@@ -6299,7 +6300,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A13" s="4" t="s">
         <v>75</v>
       </c>
@@ -6319,7 +6320,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A14" s="4" t="s">
         <v>72</v>
       </c>
@@ -6339,7 +6340,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A15" s="4" t="s">
         <v>123</v>
       </c>
@@ -6362,7 +6363,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A16" s="4" t="s">
         <v>97</v>
       </c>
@@ -6385,7 +6386,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A17" s="4"/>
       <c r="B17" s="5"/>
       <c r="C17" s="5"/>
@@ -6394,7 +6395,7 @@
       <c r="F17" s="4"/>
       <c r="G17" s="5"/>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A18" s="4" t="s">
         <v>1</v>
       </c>
@@ -6414,7 +6415,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A19" s="4" t="s">
         <v>166</v>
       </c>
@@ -6437,7 +6438,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A20" s="4"/>
       <c r="B20" s="5"/>
       <c r="C20" s="5"/>
@@ -6446,7 +6447,7 @@
       <c r="F20" s="4"/>
       <c r="G20" s="5"/>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A21" s="4" t="s">
         <v>97</v>
       </c>
@@ -6469,7 +6470,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A22" s="4" t="s">
         <v>123</v>
       </c>
@@ -6492,7 +6493,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A23" s="4" t="s">
         <v>147</v>
       </c>
@@ -6515,7 +6516,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="25" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A25" s="4" t="s">
         <v>97</v>
       </c>
@@ -6538,7 +6540,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A26" s="4" t="s">
         <v>147</v>
       </c>
@@ -6561,7 +6563,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A27" s="4" t="s">
         <v>150</v>
       </c>
@@ -6584,7 +6586,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A28" s="4" t="s">
         <v>166</v>
       </c>
@@ -6607,7 +6609,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A29" s="4" t="s">
         <v>168</v>
       </c>
@@ -6630,7 +6632,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A30" s="4" t="s">
         <v>166</v>
       </c>
@@ -6653,7 +6655,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="32" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A32" s="4" t="s">
         <v>94</v>
       </c>
@@ -6722,7 +6725,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35" s="4"/>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -6731,7 +6734,7 @@
       <c r="F35" s="4"/>
       <c r="G35" s="6"/>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
         <v>97</v>
       </c>
@@ -6754,7 +6757,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
         <v>123</v>
       </c>
@@ -6777,7 +6780,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
         <v>1</v>
       </c>
@@ -6797,7 +6801,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
         <v>89</v>
       </c>
@@ -6820,7 +6824,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41" s="4" t="s">
         <v>123</v>
       </c>
@@ -6843,7 +6847,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43" s="4" t="s">
         <v>167</v>
       </c>
@@ -6866,7 +6871,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44" s="4" t="s">
         <v>168</v>
       </c>
@@ -6889,7 +6894,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46" s="4" t="s">
         <v>1</v>
       </c>
@@ -6909,7 +6915,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:7" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="7" t="s">
         <v>85</v>
       </c>
@@ -6929,7 +6935,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="48" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48" s="4" t="s">
         <v>94</v>
       </c>
@@ -6952,7 +6958,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="49" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49" s="4" t="s">
         <v>159</v>
       </c>
@@ -6975,7 +6981,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="50" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50" s="4" t="s">
         <v>166</v>
       </c>
@@ -6998,7 +7004,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51" s="29"/>
       <c r="B51" s="28"/>
       <c r="C51" s="28"/>
@@ -7007,7 +7013,7 @@
       <c r="F51" s="29"/>
       <c r="G51" s="28"/>
     </row>
-    <row r="52" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52" s="4" t="s">
         <v>1</v>
       </c>
@@ -7027,7 +7033,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="53" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53" s="4" t="s">
         <v>71</v>
       </c>
@@ -7047,7 +7053,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="54" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54" s="4" t="s">
         <v>80</v>
       </c>
@@ -7067,7 +7073,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="55" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55" s="4" t="s">
         <v>160</v>
       </c>
@@ -7090,7 +7096,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="56" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56" s="4" t="s">
         <v>162</v>
       </c>
@@ -7113,8 +7119,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="57" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4"/>
-    <row r="58" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="58" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>1</v>
       </c>
@@ -7134,7 +7140,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="59" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59" s="4" t="s">
         <v>97</v>
       </c>
@@ -7157,7 +7163,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61" s="4" t="s">
         <v>1</v>
       </c>
@@ -7177,7 +7184,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="62" spans="1:7" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:7" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="7" t="s">
         <v>114</v>
       </c>
@@ -7200,7 +7207,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="63" spans="1:7" ht="15" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63" s="4" t="s">
         <v>115</v>
       </c>
@@ -7223,7 +7230,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="64" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64" s="4" t="s">
         <v>123</v>
       </c>
@@ -7246,7 +7253,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65" s="4" t="s">
         <v>123</v>
       </c>
@@ -7269,7 +7276,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66" s="4" t="s">
         <v>145</v>
       </c>
@@ -7292,7 +7299,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67" s="4" t="s">
         <v>146</v>
       </c>
@@ -7315,7 +7322,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68" s="4" t="s">
         <v>150</v>
       </c>
@@ -7338,7 +7345,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69" s="4" t="s">
         <v>147</v>
       </c>
@@ -7361,7 +7368,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70" s="4" t="s">
         <v>162</v>
       </c>
@@ -7384,7 +7391,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71" s="4"/>
       <c r="B71" s="5"/>
       <c r="C71" s="5"/>
@@ -7393,7 +7400,7 @@
       <c r="F71" s="4"/>
       <c r="G71" s="5"/>
     </row>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72" s="4" t="s">
         <v>113</v>
       </c>
@@ -7416,7 +7423,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="4" t="s">
         <v>1</v>
       </c>
@@ -7436,7 +7443,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="75" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75" s="4" t="s">
         <v>94</v>
       </c>
@@ -7459,7 +7467,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76" s="4" t="s">
         <v>111</v>
       </c>
@@ -7482,7 +7490,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77" s="4" t="s">
         <v>123</v>
       </c>
@@ -7505,7 +7513,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78" s="4" t="s">
         <v>158</v>
       </c>
@@ -7528,7 +7536,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79" s="4" t="s">
         <v>162</v>
       </c>
@@ -7551,7 +7559,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="81" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="81" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81" s="4" t="s">
         <v>1</v>
       </c>
@@ -7571,7 +7580,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="82" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82" s="4" t="s">
         <v>115</v>
       </c>
@@ -7594,7 +7603,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="84" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="84" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84" s="4" t="s">
         <v>1</v>
       </c>
@@ -7614,7 +7624,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="85" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85" s="4" t="s">
         <v>123</v>
       </c>
@@ -7637,7 +7647,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="86" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86" s="4" t="s">
         <v>81</v>
       </c>
@@ -7657,7 +7667,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="88" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="88" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88" s="4" t="s">
         <v>1</v>
       </c>
@@ -7677,7 +7688,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="89" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89" s="4" t="s">
         <v>123</v>
       </c>
@@ -7700,7 +7711,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="90" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90" s="4" t="s">
         <v>162</v>
       </c>
@@ -7723,7 +7734,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="91" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91" s="4"/>
       <c r="B91" s="5"/>
       <c r="C91" s="5"/>
@@ -7732,7 +7743,8 @@
       <c r="F91" s="4"/>
       <c r="G91" s="5"/>
     </row>
-    <row r="93" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="93" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93" s="4" t="s">
         <v>140</v>
       </c>
@@ -7755,7 +7767,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="94" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94" s="4" t="s">
         <v>144</v>
       </c>
@@ -7778,7 +7790,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="96" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="96" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96" s="4" t="s">
         <v>166</v>
       </c>
@@ -7801,7 +7814,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="97" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97" s="4" t="s">
         <v>162</v>
       </c>
@@ -7824,7 +7837,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="98" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98" s="4" t="s">
         <v>162</v>
       </c>
@@ -7847,7 +7860,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="99" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99" s="4" t="s">
         <v>161</v>
       </c>
@@ -7870,7 +7883,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="101" spans="1:7" ht="29" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="101" spans="1:7" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101" s="30" t="s">
         <v>172</v>
       </c>
@@ -7890,7 +7904,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="102" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102" s="31" t="s">
         <v>178</v>
       </c>
@@ -7910,7 +7924,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="103" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103" s="31" t="s">
         <v>178</v>
       </c>
@@ -7930,7 +7944,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="104" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104" s="31" t="s">
         <v>178</v>
       </c>
@@ -7950,7 +7964,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="105" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="31" t="s">
         <v>178</v>
       </c>
@@ -7970,7 +7984,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="106" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="31" t="s">
         <v>178</v>
       </c>
@@ -7990,7 +8004,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="107" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="31" t="s">
         <v>178</v>
       </c>
@@ -8010,7 +8024,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="108" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="31" t="s">
         <v>178</v>
       </c>
@@ -8030,7 +8044,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="109" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A109" s="31" t="s">
         <v>178</v>
       </c>
@@ -8050,7 +8064,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="110" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A110" s="31" t="s">
         <v>178</v>
       </c>
@@ -8070,7 +8084,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="111" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A111" s="31" t="s">
         <v>178</v>
       </c>
@@ -8090,7 +8104,7 @@
         <v>210</v>
       </c>
     </row>
-    <row r="112" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A112" s="31" t="s">
         <v>178</v>
       </c>
@@ -8110,7 +8124,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A113" s="31" t="s">
         <v>178</v>
       </c>
@@ -8130,7 +8144,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A114" s="31" t="s">
         <v>178</v>
       </c>
@@ -8150,7 +8164,7 @@
         <v>219</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A115" s="31" t="s">
         <v>178</v>
       </c>
@@ -8170,7 +8184,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A116" s="31" t="s">
         <v>178</v>
       </c>
@@ -8190,7 +8204,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A117" s="31" t="s">
         <v>178</v>
       </c>
@@ -8210,7 +8224,7 @@
         <v>228</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A118" s="31" t="s">
         <v>178</v>
       </c>
@@ -8230,7 +8244,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A119" s="31" t="s">
         <v>178</v>
       </c>
@@ -8250,7 +8264,7 @@
         <v>234</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A120" s="31" t="s">
         <v>178</v>
       </c>
@@ -8270,7 +8284,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A121" s="31" t="s">
         <v>178</v>
       </c>
@@ -8290,7 +8304,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A122" s="31" t="s">
         <v>178</v>
       </c>
@@ -8310,7 +8324,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A123" s="31" t="s">
         <v>178</v>
       </c>
@@ -8330,7 +8344,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A124" s="31" t="s">
         <v>178</v>
       </c>
@@ -8350,7 +8364,7 @@
         <v>251</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A125" s="31" t="s">
         <v>178</v>
       </c>
@@ -8370,7 +8384,7 @@
         <v>254</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A126" s="31" t="s">
         <v>178</v>
       </c>
@@ -8390,7 +8404,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A127" s="31" t="s">
         <v>178</v>
       </c>
@@ -8410,7 +8424,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A128" s="31" t="s">
         <v>178</v>
       </c>
@@ -8430,7 +8444,7 @@
         <v>263</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A129" s="31" t="s">
         <v>178</v>
       </c>
@@ -8450,7 +8464,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A130" s="31" t="s">
         <v>178</v>
       </c>
@@ -8470,7 +8484,7 @@
         <v>271</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A131" s="31" t="s">
         <v>178</v>
       </c>
@@ -8490,7 +8504,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A132" s="31" t="s">
         <v>178</v>
       </c>
@@ -8510,7 +8524,7 @@
         <v>279</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="133" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A133" s="31" t="s">
         <v>178</v>
       </c>
@@ -8530,7 +8544,7 @@
         <v>283</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="134" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A134" s="31" t="s">
         <v>178</v>
       </c>
@@ -8550,7 +8564,7 @@
         <v>286</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="135" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A135" s="31" t="s">
         <v>178</v>
       </c>
@@ -8570,7 +8584,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="136" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A136" s="31" t="s">
         <v>178</v>
       </c>
@@ -8590,7 +8604,7 @@
         <v>292</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="137" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A137" s="31" t="s">
         <v>178</v>
       </c>
@@ -8610,7 +8624,7 @@
         <v>295</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="138" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A138" s="31" t="s">
         <v>178</v>
       </c>
@@ -8630,7 +8644,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="139" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A139" s="31" t="s">
         <v>178</v>
       </c>
@@ -8650,7 +8664,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="140" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A140" s="31" t="s">
         <v>178</v>
       </c>
@@ -8670,7 +8684,7 @@
         <v>305</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="141" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A141" s="31" t="s">
         <v>178</v>
       </c>
@@ -8690,7 +8704,7 @@
         <v>309</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="142" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A142" s="31" t="s">
         <v>178</v>
       </c>
@@ -8710,7 +8724,7 @@
         <v>313</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="143" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A143" s="31" t="s">
         <v>178</v>
       </c>
@@ -8730,7 +8744,7 @@
         <v>317</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="144" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A144" s="31" t="s">
         <v>178</v>
       </c>
@@ -8750,7 +8764,7 @@
         <v>244</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="145" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A145" s="31" t="s">
         <v>178</v>
       </c>
@@ -8770,7 +8784,7 @@
         <v>323</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="146" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A146" s="36" t="s">
         <v>324</v>
       </c>
@@ -8790,7 +8804,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="147" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A147" s="36" t="s">
         <v>324</v>
       </c>
@@ -8810,7 +8824,7 @@
         <v>330</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="148" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A148" s="36" t="s">
         <v>324</v>
       </c>
@@ -8830,7 +8844,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="149" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A149" s="36" t="s">
         <v>324</v>
       </c>
@@ -8850,7 +8864,7 @@
         <v>198</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="150" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A150" s="36" t="s">
         <v>324</v>
       </c>
@@ -8870,7 +8884,7 @@
         <v>338</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="151" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A151" s="36" t="s">
         <v>324</v>
       </c>
@@ -8890,7 +8904,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="152" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A152" s="36" t="s">
         <v>324</v>
       </c>
@@ -8910,7 +8924,7 @@
         <v>248</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="153" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A153" s="36" t="s">
         <v>324</v>
       </c>
@@ -8930,7 +8944,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="154" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A154" s="36" t="s">
         <v>324</v>
       </c>
@@ -8950,7 +8964,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="155" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A155" s="36" t="s">
         <v>324</v>
       </c>
@@ -8970,7 +8984,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="156" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A156" s="36" t="s">
         <v>324</v>
       </c>
@@ -8990,7 +9004,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="157" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A157" s="36" t="s">
         <v>324</v>
       </c>
@@ -9010,7 +9024,7 @@
         <v>361</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="158" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A158" s="36" t="s">
         <v>324</v>
       </c>
@@ -9030,7 +9044,7 @@
         <v>364</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="159" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A159" s="36" t="s">
         <v>324</v>
       </c>
@@ -9050,7 +9064,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="160" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A160" s="36" t="s">
         <v>324</v>
       </c>
@@ -9070,7 +9084,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="161" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A161" s="36" t="s">
         <v>324</v>
       </c>
@@ -9090,7 +9104,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="162" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A162" s="36" t="s">
         <v>324</v>
       </c>
@@ -9110,7 +9124,7 @@
         <v>371</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="163" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A163" s="36" t="s">
         <v>324</v>
       </c>
@@ -9130,7 +9144,7 @@
         <v>379</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="164" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A164" s="36" t="s">
         <v>324</v>
       </c>
@@ -9150,7 +9164,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="165" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A165" s="36" t="s">
         <v>324</v>
       </c>
@@ -9170,7 +9184,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="166" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A166" s="36" t="s">
         <v>324</v>
       </c>
@@ -9190,7 +9204,7 @@
         <v>388</v>
       </c>
     </row>
-    <row r="167" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="167" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A167" s="36" t="s">
         <v>324</v>
       </c>
@@ -9210,7 +9224,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="168" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="168" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A168" s="36" t="s">
         <v>324</v>
       </c>
@@ -9230,7 +9244,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="169" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="169" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A169" s="36" t="s">
         <v>324</v>
       </c>
@@ -9250,7 +9264,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="170" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="170" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A170" s="36" t="s">
         <v>324</v>
       </c>
@@ -9330,7 +9344,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="174" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="174" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A174" s="36" t="s">
         <v>324</v>
       </c>
@@ -9350,7 +9364,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="175" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="175" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A175" s="36" t="s">
         <v>324</v>
       </c>
@@ -9370,7 +9384,7 @@
         <v>416</v>
       </c>
     </row>
-    <row r="176" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="176" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A176" s="36" t="s">
         <v>324</v>
       </c>
@@ -9390,7 +9404,7 @@
         <v>419</v>
       </c>
     </row>
-    <row r="177" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="177" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A177" s="41" t="s">
         <v>420</v>
       </c>
@@ -9410,7 +9424,7 @@
         <v>391</v>
       </c>
     </row>
-    <row r="178" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="178" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A178" s="41" t="s">
         <v>420</v>
       </c>
@@ -9430,7 +9444,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="179" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="179" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A179" s="41" t="s">
         <v>420</v>
       </c>
@@ -9450,7 +9464,7 @@
         <v>425</v>
       </c>
     </row>
-    <row r="180" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="180" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A180" s="41" t="s">
         <v>420</v>
       </c>
@@ -9470,7 +9484,7 @@
         <v>431</v>
       </c>
     </row>
-    <row r="181" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="181" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A181" s="41" t="s">
         <v>420</v>
       </c>
@@ -9490,7 +9504,7 @@
         <v>435</v>
       </c>
     </row>
-    <row r="182" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="182" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A182" s="41" t="s">
         <v>420</v>
       </c>
@@ -9510,7 +9524,7 @@
         <v>438</v>
       </c>
     </row>
-    <row r="183" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="183" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A183" s="41" t="s">
         <v>420</v>
       </c>
@@ -9530,7 +9544,7 @@
         <v>442</v>
       </c>
     </row>
-    <row r="184" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="184" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A184" s="41" t="s">
         <v>420</v>
       </c>
@@ -9550,7 +9564,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="185" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="185" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A185" s="41" t="s">
         <v>420</v>
       </c>
@@ -9570,7 +9584,7 @@
         <v>447</v>
       </c>
     </row>
-    <row r="186" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="186" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A186" s="46" t="s">
         <v>448</v>
       </c>
@@ -9590,7 +9604,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="187" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="187" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A187" s="46" t="s">
         <v>448</v>
       </c>
@@ -9610,7 +9624,7 @@
         <v>454</v>
       </c>
     </row>
-    <row r="188" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="188" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A188" s="46" t="s">
         <v>448</v>
       </c>
@@ -9690,7 +9704,7 @@
         <v>461</v>
       </c>
     </row>
-    <row r="192" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="192" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A192" s="46" t="s">
         <v>448</v>
       </c>
@@ -9710,7 +9724,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="193" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="193" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A193" s="46" t="s">
         <v>448</v>
       </c>
@@ -9730,7 +9744,7 @@
         <v>394</v>
       </c>
     </row>
-    <row r="194" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="194" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A194" s="46" t="s">
         <v>448</v>
       </c>
@@ -9750,7 +9764,7 @@
         <v>472</v>
       </c>
     </row>
-    <row r="195" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="195" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="A195" s="46" t="s">
         <v>448</v>
       </c>
@@ -9770,7 +9784,8 @@
         <v>475</v>
       </c>
     </row>
-    <row r="197" spans="1:6" ht="29" x14ac:dyDescent="0.35">
+    <row r="196" spans="1:6" hidden="1" x14ac:dyDescent="0.35"/>
+    <row r="197" spans="1:6" ht="29" hidden="1" x14ac:dyDescent="0.35">
       <c r="B197" s="51" t="s">
         <v>173</v>
       </c>
@@ -9787,7 +9802,7 @@
         <v>479</v>
       </c>
     </row>
-    <row r="198" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="198" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B198" s="52" t="s">
         <v>320</v>
       </c>
@@ -9804,7 +9819,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="199" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="199" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B199" s="57" t="s">
         <v>314</v>
       </c>
@@ -9821,7 +9836,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="200" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="200" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B200" s="52" t="s">
         <v>306</v>
       </c>
@@ -9838,7 +9853,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="201" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="201" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B201" s="57" t="s">
         <v>487</v>
       </c>
@@ -9855,7 +9870,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="202" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="202" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B202" s="52" t="s">
         <v>487</v>
       </c>
@@ -9872,7 +9887,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="203" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="203" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B203" s="57" t="s">
         <v>492</v>
       </c>
@@ -9889,7 +9904,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="204" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="204" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B204" s="52" t="s">
         <v>492</v>
       </c>
@@ -9906,7 +9921,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="205" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="205" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B205" s="57" t="s">
         <v>492</v>
       </c>
@@ -9923,7 +9938,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="206" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="206" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B206" s="52" t="s">
         <v>492</v>
       </c>
@@ -9940,7 +9955,7 @@
         <v>238</v>
       </c>
     </row>
-    <row r="207" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="207" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B207" s="57" t="s">
         <v>492</v>
       </c>
@@ -9957,7 +9972,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="208" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="208" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B208" s="52" t="s">
         <v>503</v>
       </c>
@@ -9974,7 +9989,7 @@
         <v>506</v>
       </c>
     </row>
-    <row r="209" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="209" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B209" s="57" t="s">
         <v>503</v>
       </c>
@@ -9991,7 +10006,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="210" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="210" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B210" s="52" t="s">
         <v>503</v>
       </c>
@@ -10008,7 +10023,7 @@
         <v>509</v>
       </c>
     </row>
-    <row r="211" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="211" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B211" s="57" t="s">
         <v>512</v>
       </c>
@@ -10025,7 +10040,7 @@
         <v>515</v>
       </c>
     </row>
-    <row r="212" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="212" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B212" s="57" t="s">
         <v>516</v>
       </c>
@@ -10042,7 +10057,7 @@
         <v>519</v>
       </c>
     </row>
-    <row r="213" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="213" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B213" s="57" t="s">
         <v>276</v>
       </c>
@@ -10059,7 +10074,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="214" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="214" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B214" s="52" t="s">
         <v>272</v>
       </c>
@@ -10076,7 +10091,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="215" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="215" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B215" s="57" t="s">
         <v>302</v>
       </c>
@@ -10093,7 +10108,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="216" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="216" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B216" s="52" t="s">
         <v>302</v>
       </c>
@@ -10110,7 +10125,7 @@
         <v>527</v>
       </c>
     </row>
-    <row r="217" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="217" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B217" s="57" t="s">
         <v>530</v>
       </c>
@@ -10127,7 +10142,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="218" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="218" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B218" s="52" t="s">
         <v>530</v>
       </c>
@@ -10144,7 +10159,7 @@
         <v>535</v>
       </c>
     </row>
-    <row r="219" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="219" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B219" s="57" t="s">
         <v>223</v>
       </c>
@@ -10161,7 +10176,7 @@
         <v>538</v>
       </c>
     </row>
-    <row r="220" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="220" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B220" s="52" t="s">
         <v>223</v>
       </c>
@@ -10178,7 +10193,7 @@
         <v>541</v>
       </c>
     </row>
-    <row r="221" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="221" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B221" s="57" t="s">
         <v>179</v>
       </c>
@@ -10195,7 +10210,7 @@
         <v>544</v>
       </c>
     </row>
-    <row r="222" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="222" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B222" s="52" t="s">
         <v>179</v>
       </c>
@@ -10212,7 +10227,7 @@
         <v>207</v>
       </c>
     </row>
-    <row r="223" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="223" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B223" s="57" t="s">
         <v>179</v>
       </c>
@@ -10229,7 +10244,7 @@
         <v>549</v>
       </c>
     </row>
-    <row r="224" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="224" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B224" s="52" t="s">
         <v>280</v>
       </c>
@@ -10246,7 +10261,7 @@
         <v>552</v>
       </c>
     </row>
-    <row r="225" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="225" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B225" s="57" t="s">
         <v>211</v>
       </c>
@@ -10263,7 +10278,7 @@
         <v>555</v>
       </c>
     </row>
-    <row r="226" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="226" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B226" s="52" t="s">
         <v>211</v>
       </c>
@@ -10280,7 +10295,7 @@
         <v>558</v>
       </c>
     </row>
-    <row r="227" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="227" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B227" s="57" t="s">
         <v>339</v>
       </c>
@@ -10297,7 +10312,7 @@
         <v>561</v>
       </c>
     </row>
-    <row r="228" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="228" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B228" s="52" t="s">
         <v>204</v>
       </c>
@@ -10314,7 +10329,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="229" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="229" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B229" s="57" t="s">
         <v>204</v>
       </c>
@@ -10331,7 +10346,7 @@
         <v>567</v>
       </c>
     </row>
-    <row r="230" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="230" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B230" s="52" t="s">
         <v>204</v>
       </c>
@@ -10399,7 +10414,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="234" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="234" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B234" s="52" t="s">
         <v>343</v>
       </c>
@@ -10416,7 +10431,7 @@
         <v>580</v>
       </c>
     </row>
-    <row r="235" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="235" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B235" s="57" t="s">
         <v>235</v>
       </c>
@@ -10433,7 +10448,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="236" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="236" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B236" s="52" t="s">
         <v>467</v>
       </c>
@@ -10450,7 +10465,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="237" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="237" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B237" s="57" t="s">
         <v>467</v>
       </c>
@@ -10467,7 +10482,7 @@
         <v>588</v>
       </c>
     </row>
-    <row r="238" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="238" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B238" s="52" t="s">
         <v>467</v>
       </c>
@@ -10484,7 +10499,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="239" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="239" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B239" s="57" t="s">
         <v>195</v>
       </c>
@@ -10501,7 +10516,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="240" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="240" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B240" s="52" t="s">
         <v>195</v>
       </c>
@@ -10518,7 +10533,7 @@
         <v>475</v>
       </c>
     </row>
-    <row r="241" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="241" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B241" s="57" t="s">
         <v>195</v>
       </c>
@@ -10535,7 +10550,7 @@
         <v>591</v>
       </c>
     </row>
-    <row r="242" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="242" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B242" s="52" t="s">
         <v>314</v>
       </c>
@@ -10552,7 +10567,7 @@
         <v>564</v>
       </c>
     </row>
-    <row r="243" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="243" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B243" s="57" t="s">
         <v>343</v>
       </c>
@@ -10569,7 +10584,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="244" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="244" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B244" s="52" t="s">
         <v>343</v>
       </c>
@@ -10586,7 +10601,7 @@
         <v>583</v>
       </c>
     </row>
-    <row r="245" spans="2:6" x14ac:dyDescent="0.35">
+    <row r="245" spans="2:6" hidden="1" x14ac:dyDescent="0.35">
       <c r="B245" s="57" t="s">
         <v>343</v>
       </c>
@@ -10604,7 +10619,14 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="B1:B245" xr:uid="{BDEAB589-59D4-402D-A28C-AA7262E65C2C}"/>
+  <autoFilter ref="B1:B245" xr:uid="{BDEAB589-59D4-402D-A28C-AA7262E65C2C}">
+    <filterColumn colId="0">
+      <filters>
+        <filter val="GRSE"/>
+        <filter val="GRSEEQ"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Order files updated upto 12 aug 2026 Wednesday
</commit_message>
<xml_diff>
--- a/ORDER_MGMT/regular_order_mgmt/PENDING_ORDERS_REPOSITORY_FILES/Result_Executed_OrderBook_14to24july2026.xlsx
+++ b/ORDER_MGMT/regular_order_mgmt/PENDING_ORDERS_REPOSITORY_FILES/Result_Executed_OrderBook_14to24july2026.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\python\stocks\ORDER_MGMT\regular_order_mgmt\PENDING_ORDERS_REPOSITORY_FILES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B6E68CC-7D67-4239-A6E4-FD108EF93969}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5637B71-EE97-4617-8FC1-54CDF90862FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -6679,7 +6679,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
         <v>149</v>
       </c>
@@ -6725,7 +6725,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A35" s="4"/>
       <c r="B35" s="6"/>
       <c r="C35" s="6"/>
@@ -6734,7 +6734,7 @@
       <c r="F35" s="4"/>
       <c r="G35" s="6"/>
     </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A36" s="4" t="s">
         <v>97</v>
       </c>
@@ -6757,7 +6757,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A37" s="4" t="s">
         <v>123</v>
       </c>
@@ -6780,8 +6780,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="39" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A39" s="4" t="s">
         <v>1</v>
       </c>
@@ -6801,7 +6801,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A40" s="4" t="s">
         <v>89</v>
       </c>
@@ -6824,7 +6824,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A41" s="4" t="s">
         <v>123</v>
       </c>
@@ -6847,8 +6847,8 @@
         <v>49</v>
       </c>
     </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.35"/>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35"/>
+    <row r="43" spans="1:7" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A43" s="4" t="s">
         <v>167</v>
       </c>
@@ -8504,7 +8504,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="132" spans="1:6" hidden="1" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:6" ht="15" hidden="1" thickTop="1" x14ac:dyDescent="0.35">
       <c r="A132" s="31" t="s">
         <v>178</v>
       </c>

</xml_diff>

<commit_message>
Orders fully updated upto 14 aug 2026 Friday
</commit_message>
<xml_diff>
--- a/ORDER_MGMT/regular_order_mgmt/PENDING_ORDERS_REPOSITORY_FILES/Result_Executed_OrderBook_14to24july2026.xlsx
+++ b/ORDER_MGMT/regular_order_mgmt/PENDING_ORDERS_REPOSITORY_FILES/Result_Executed_OrderBook_14to24july2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\python\stocks\ORDER_MGMT\regular_order_mgmt\PENDING_ORDERS_REPOSITORY_FILES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5637B71-EE97-4617-8FC1-54CDF90862FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8BEF295D-C7C7-4D24-B451-DB82322141B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="All_Backups" sheetId="2" r:id="rId1"/>
@@ -6679,7 +6679,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="33" spans="1:7" thickTop="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A33" s="4" t="s">
         <v>149</v>
       </c>
@@ -10648,7 +10648,7 @@
       </c>
       <c r="C1" s="23">
         <f>SUM(C3:C30000)/SUM(A3:A300000)</f>
-        <v>1150.5</v>
+        <v>2089</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.35">
@@ -10660,39 +10660,35 @@
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A3" s="5">
-        <v>10</v>
-      </c>
-      <c r="B3" s="4">
-        <v>1140</v>
+      <c r="A3">
+        <v>5</v>
+      </c>
+      <c r="B3">
+        <v>2114</v>
       </c>
       <c r="C3">
         <f>B3*A3</f>
-        <v>11400</v>
+        <v>10570</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A4" s="5">
-        <v>5</v>
-      </c>
-      <c r="B4" s="4">
-        <v>1152</v>
+      <c r="A4">
+        <v>5</v>
+      </c>
+      <c r="B4">
+        <v>2064</v>
       </c>
       <c r="C4">
         <f>B4*A4</f>
-        <v>5760</v>
+        <v>10320</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
-      <c r="A5" s="5">
-        <v>5</v>
-      </c>
-      <c r="B5" s="4">
-        <v>1170</v>
-      </c>
+      <c r="A5" s="5"/>
+      <c r="B5" s="4"/>
       <c r="C5">
         <f t="shared" ref="C5:C18" si="0">B5*A5</f>
-        <v>5850</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">

</xml_diff>